<commit_message>
atualização dos requisitos fn e rnf
</commit_message>
<xml_diff>
--- a/REQUISITOS FUNCIONAI E NÃO FUNCIONAIS DO PETPOP.xlsx
+++ b/REQUISITOS FUNCIONAI E NÃO FUNCIONAIS DO PETPOP.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2026\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2026\Desktop\petpops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B86B31FC-45EF-4E47-A53A-BA036E81475C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3715791C-0606-43FE-AD9A-39EA4CE7EBDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8693B3CC-EAAC-4797-85BA-6A94D83F9FE7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t>ID</t>
   </si>
@@ -165,6 +165,18 @@
   </si>
   <si>
     <t>INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>RNF-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O SITE DEVE TER O CONTADO DE OUTRAS CLINICAS </t>
+  </si>
+  <si>
+    <t>RNF-07</t>
+  </si>
+  <si>
+    <t>O SITE DEVE TER UM CHAT BOT  24 HORAS PARA  DUVIDAS</t>
   </si>
 </sst>
 </file>
@@ -278,19 +290,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -299,12 +311,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -641,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D502D947-C4EA-438D-948E-6F249F6EE7BD}">
-  <dimension ref="D3:H24"/>
+  <dimension ref="D4:G24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="57.109375" bestFit="1" customWidth="1"/>
@@ -649,252 +655,255 @@
     <col min="7" max="7" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D4" s="7" t="s">
+    <row r="4" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D5" s="10" t="s">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D6" s="4" t="s">
+    </row>
+    <row r="6" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D7" s="4" t="s">
+    </row>
+    <row r="7" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D8" s="4" t="s">
+    </row>
+    <row r="8" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D9" s="4" t="s">
+    </row>
+    <row r="9" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D10" s="4" t="s">
+    </row>
+    <row r="10" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D11" s="4" t="s">
+    </row>
+    <row r="11" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D14" s="7" t="s">
+    </row>
+    <row r="12" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="9"/>
-    </row>
-    <row r="15" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D15" s="10" t="s">
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
+    </row>
+    <row r="15" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D15" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="G15" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D16" s="4" t="s">
+    <row r="16" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="D21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
+      <c r="D22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="23" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
     </row>
     <row r="24" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
correção dos requisitos funcionais e não funcionais
</commit_message>
<xml_diff>
--- a/REQUISITOS FUNCIONAI E NÃO FUNCIONAIS DO PETPOP.xlsx
+++ b/REQUISITOS FUNCIONAI E NÃO FUNCIONAIS DO PETPOP.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2026\Desktop\petpops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2026\Desktop\PATINHAS_FELIZES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3715791C-0606-43FE-AD9A-39EA4CE7EBDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4E77E8-89AC-449B-8EA7-C975DB8827CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8693B3CC-EAAC-4797-85BA-6A94D83F9FE7}"/>
   </bookViews>
@@ -86,9 +86,6 @@
     <t>O SITE DEVE CONTER PAGINA HOME</t>
   </si>
   <si>
-    <t>O SITE DEVE CONTER UM PAGINA DE CANCELAMENTO</t>
-  </si>
-  <si>
     <t>REQUISITOS NÃO FUNCIONAIS</t>
   </si>
   <si>
@@ -177,6 +174,9 @@
   </si>
   <si>
     <t>O SITE DEVE TER UM CHAT BOT  24 HORAS PARA  DUVIDAS</t>
+  </si>
+  <si>
+    <t>O SITE DEVE CONTER UM BOTÃO DE CANCELAMENTO</t>
   </si>
 </sst>
 </file>
@@ -674,7 +674,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
@@ -682,13 +682,13 @@
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
@@ -696,13 +696,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
@@ -710,13 +710,13 @@
         <v>4</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
@@ -724,13 +724,13 @@
         <v>5</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
@@ -738,13 +738,13 @@
         <v>6</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
@@ -752,13 +752,13 @@
         <v>7</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.3">
@@ -775,7 +775,7 @@
     </row>
     <row r="14" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D14" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
@@ -786,111 +786,111 @@
         <v>0</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>1</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D17" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D18" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="G21" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="G22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="4:7" x14ac:dyDescent="0.3">

</xml_diff>